<commit_message>
feat: Ban Mong - chot 18.240 tam pin; thiet ke so bo dau coc, dai coc doi, tai neo de
- So tam pin 18.240 da chot (Chu dau tu 22/10/2026)
- twinPileCap.ts: dai BTCT noi 2 coc D350 (uon, cat, xoan, neo thep coc) + test
- shorePileHead.ts: them goc cap (thanh phan nho) va gioi han chieu dai thep neo
  cho tai neo mat de; khong truyen thi ket qua nhu cu
- Bang neo Ban Mong: dau coc, dai coc doi, tai neo de lay tu thiet ke (sheet
  KiemTra_DauCoc_De), Huoi Vanh giu nguyen order 15/10

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/docs_ban_mong/HOBANMONG_THONG_KE_VAT_TU_BE_PIN.xlsx
+++ b/public/docs_ban_mong/HOBANMONG_THONG_KE_VAT_TU_BE_PIN.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nhatm\AppData\Local\Temp\claude\E--Out-Job-Chu-Giap-Web-t-nh-neo-b-\4941c4bc-fff6-410b-95cf-e91fd3b09d53\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6A37C7F5-4940-444B-B49C-66B8758FCE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{53A0696A-3022-49E6-9A7B-8511568AF459}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2380" yWindow="4110" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -93,7 +93,7 @@
     <t>BV</t>
   </si>
   <si>
-    <t>Tổng 18.240 tấm trên bản vẽ 22/10; Pre-FS và web: 16.892 tấm (xem DoiChieu_MatBang)</t>
+    <t>ĐÃ CHỐT 18.240 tấm (Chủ đầu tư 22/10/2026), theo bảng từng tờ; Pre-FS cũ ghi 16.892 tấm</t>
   </si>
   <si>
     <t>Inverter SG-510HX</t>
@@ -1632,7 +1632,7 @@
     <t>ĐỐI CHIẾU TỪNG TỜ CT-BP (22/10/2026) VỚI MẶT BẰNG BÈ MÀ WEB DÙNG TÍNH NEO (nhập từ tờ MB-B01-01)</t>
   </si>
   <si>
-    <t>Đường bao bè đo trên ảnh từng tờ CT-BP (tỷ lệ in trên tờ, gồm cả mép phao nên rộng hơn 1–2 m); mặt bằng trên web lấy đường bao bè của tờ MB-B01-01. Số tấm pin trên web lấy đúng bảng từng tờ (Pre-FS ghi 16.892 tấm, bản vẽ 22/10 có 18.240 tấm).</t>
+    <t>Đường bao bè đo trên ảnh từng tờ CT-BP (tỷ lệ in trên tờ, gồm cả mép phao nên rộng hơn 1–2 m); mặt bằng trên web lấy đường bao bè của tờ MB-B01-01. Số tấm pin trên web lấy đúng bảng từng tờ — ĐÃ CHỐT 18.240 tấm (Pre-FS cũ ghi 16.892).</t>
   </si>
   <si>
     <t>Tỷ lệ tờ</t>
@@ -1950,7 +1950,7 @@
     <t>Mặt bằng neo (số dây, vị trí bích) là của web, tính trên mặt bằng bè 22/10/2026 (đường bao lấy từ tờ MB-B01-01, đặt về tọa độ PA2: so với PA2 chỉ BÈ 4 và BÈ 6 đổi hình). Đường bao đo trên từng tờ CT-BP rộng hơn 1–2 m vì gồm cả mép phao (sheet DoiChieu_MatBang).</t>
   </si>
   <si>
-    <t>Tổng tấm pin trên bản vẽ 18.240 tấm (13,5 MWp với tấm 740 Wp), khác Pre-FS 16.892 tấm (12,5 MWp). Tờ BÈ 2 có 1 dải 28 tấm ghi chú "be 1"; BÈ 4 ghi 80,43 string (2.252 tấm không chia hết cho 28). Cần thiết kế điện xác nhận.</t>
+    <t>Số tấm pin ĐÃ CHỐT 18.240 tấm (Chủ đầu tư 22/10/2026; 13,5 MWp với tấm 740 Wp — Pre-FS cũ ghi 16.892 tấm, 12,5 MWp). Lực gió và lực dây trên web tính theo số tấm từng bè này. Còn để thiết kế điện xem: tờ BÈ 2 có 1 dải 28 tấm ghi chú "be 1"; BÈ 4 ghi 80,43 string (2.252 tấm không chia hết cho 28).</t>
   </si>
   <si>
     <t>Khối lượng thép theo tiết diện GIẢ ĐỊNH (C52 ≈ 2,36 kg/m; hộp 40×60×2,0 ≈ 3,01 kg/m) vì chưa có catalogue tiết diện của nhà sản xuất.</t>

</xml_diff>

<commit_message>
feat: Ban Mong - D14 (B3-D16) len coc mui dat, D15 ra bo; noi cung ho BE 3 toi 70 do
- B3-D16 coc dat tay tren mui dat (44; 147), day 46 m, khong cat day nao (planner chi thu diem bo dau tien moi huong).
- Planner: maxArcFor (lakeConfig) noi cung ho theo tung be; BE 3 70 do (engine dat 78,7 kN PES-32, troi 0,79 m).
- B3-D18 ra bo 42 m. He neo: 215 day (188 bo + 27 day) + 14 day noi, 17 de 128 m3, 68 vit.
- Ho so tao lai.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/docs_ban_mong/HOBANMONG_THONG_KE_VAT_TU_BE_PIN.xlsx
+++ b/public/docs_ban_mong/HOBANMONG_THONG_KE_VAT_TU_BE_PIN.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nhatm\AppData\Local\Temp\claude\E--Out-Job-Chu-Giap-Web-t-nh-neo-b-\6aeb2207-6b11-48a0-9210-732f1cccfe43\scratchpad\bmkc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2527E6F4-7FD8-4C3D-A1E0-8BB7AA031DD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4D5EDF0A-BABD-46BE-8738-101EE301844E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3120" yWindow="2890" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -14937,11 +14937,11 @@
         <v>2</v>
       </c>
       <c r="F124" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G124" s="11">
         <f>2*F124*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>128.51999999999998</v>
+        <v>132.21599999999998</v>
       </c>
       <c r="H124" s="7">
         <v>12</v>
@@ -15005,11 +15005,11 @@
         <v>2</v>
       </c>
       <c r="F125" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G125" s="11">
         <f>2*F125*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>128.51999999999998</v>
+        <v>132.21599999999998</v>
       </c>
       <c r="H125" s="7">
         <v>12</v>
@@ -15073,11 +15073,11 @@
         <v>2</v>
       </c>
       <c r="F126" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G126" s="11">
         <f>2*F126*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>128.51999999999998</v>
+        <v>132.21599999999998</v>
       </c>
       <c r="H126" s="7">
         <v>13</v>
@@ -15141,11 +15141,11 @@
         <v>2</v>
       </c>
       <c r="F127" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G127" s="11">
         <f>2*F127*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>128.51999999999998</v>
+        <v>132.21599999999998</v>
       </c>
       <c r="H127" s="7">
         <v>12</v>
@@ -15209,11 +15209,11 @@
         <v>4</v>
       </c>
       <c r="F128" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G128" s="11">
         <f>4*F128*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>257.03999999999996</v>
+        <v>264.43199999999996</v>
       </c>
       <c r="H128" s="7">
         <v>11</v>
@@ -15277,11 +15277,11 @@
         <v>2</v>
       </c>
       <c r="F129" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G129" s="11">
         <f>2*F129*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>128.51999999999998</v>
+        <v>132.21599999999998</v>
       </c>
       <c r="H129" s="7">
         <v>13</v>
@@ -15345,11 +15345,11 @@
         <v>1</v>
       </c>
       <c r="F130" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G130" s="11">
         <f>1*F130*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H130" s="7">
         <v>13</v>
@@ -15413,11 +15413,11 @@
         <v>1</v>
       </c>
       <c r="F131" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G131" s="11">
         <f>1*F131*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H131" s="7">
         <v>13</v>
@@ -15481,11 +15481,11 @@
         <v>1</v>
       </c>
       <c r="F132" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G132" s="11">
         <f>1*F132*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H132" s="7">
         <v>13</v>
@@ -15549,11 +15549,11 @@
         <v>1</v>
       </c>
       <c r="F133" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G133" s="11">
         <f>1*F133*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H133" s="7">
         <v>13</v>
@@ -15617,11 +15617,11 @@
         <v>1</v>
       </c>
       <c r="F134" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G134" s="11">
         <f>1*F134*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H134" s="7">
         <v>13</v>
@@ -15685,11 +15685,11 @@
         <v>1</v>
       </c>
       <c r="F135" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G135" s="11">
         <f>1*F135*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H135" s="7">
         <v>13</v>
@@ -15753,11 +15753,11 @@
         <v>1</v>
       </c>
       <c r="F136" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G136" s="11">
         <f>1*F136*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H136" s="7">
         <v>13</v>
@@ -15821,11 +15821,11 @@
         <v>1</v>
       </c>
       <c r="F137" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G137" s="11">
         <f>1*F137*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H137" s="7">
         <v>13</v>
@@ -15889,11 +15889,11 @@
         <v>1</v>
       </c>
       <c r="F138" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G138" s="11">
         <f>1*F138*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H138" s="7">
         <v>13</v>
@@ -15957,11 +15957,11 @@
         <v>1</v>
       </c>
       <c r="F139" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G139" s="11">
         <f>1*F139*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H139" s="7">
         <v>13</v>
@@ -16025,11 +16025,11 @@
         <v>1</v>
       </c>
       <c r="F140" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G140" s="11">
         <f>1*F140*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H140" s="7">
         <v>12</v>
@@ -16093,11 +16093,11 @@
         <v>1</v>
       </c>
       <c r="F141" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G141" s="11">
         <f>1*F141*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H141" s="7">
         <v>12</v>
@@ -16161,11 +16161,11 @@
         <v>1</v>
       </c>
       <c r="F142" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G142" s="11">
         <f>1*F142*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H142" s="7">
         <v>12</v>
@@ -16229,11 +16229,11 @@
         <v>1</v>
       </c>
       <c r="F143" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G143" s="11">
         <f>1*F143*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H143" s="7">
         <v>12</v>
@@ -16297,11 +16297,11 @@
         <v>1</v>
       </c>
       <c r="F144" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G144" s="11">
         <f>1*F144*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H144" s="7">
         <v>12</v>
@@ -16365,11 +16365,11 @@
         <v>1</v>
       </c>
       <c r="F145" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G145" s="11">
         <f>1*F145*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H145" s="7">
         <v>12</v>
@@ -16433,11 +16433,11 @@
         <v>1</v>
       </c>
       <c r="F146" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G146" s="11">
         <f>1*F146*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H146" s="7">
         <v>12</v>
@@ -16501,11 +16501,11 @@
         <v>1</v>
       </c>
       <c r="F147" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G147" s="11">
         <f>1*F147*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H147" s="7">
         <v>12</v>
@@ -16569,11 +16569,11 @@
         <v>1</v>
       </c>
       <c r="F148" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G148" s="11">
         <f>1*F148*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H148" s="7">
         <v>12</v>
@@ -16637,11 +16637,11 @@
         <v>1</v>
       </c>
       <c r="F149" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G149" s="11">
         <f>1*F149*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H149" s="7">
         <v>12</v>
@@ -16705,11 +16705,11 @@
         <v>1</v>
       </c>
       <c r="F150" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G150" s="11">
         <f>1*F150*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H150" s="7">
         <v>12</v>
@@ -16773,11 +16773,11 @@
         <v>1</v>
       </c>
       <c r="F151" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G151" s="11">
         <f>1*F151*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H151" s="7">
         <v>12</v>
@@ -16841,11 +16841,11 @@
         <v>1</v>
       </c>
       <c r="F152" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G152" s="11">
         <f>1*F152*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H152" s="7">
         <v>12</v>
@@ -16909,11 +16909,11 @@
         <v>1</v>
       </c>
       <c r="F153" s="7">
-        <v>76.5</v>
+        <v>78.7</v>
       </c>
       <c r="G153" s="11">
         <f>1*F153*GiaDinh!$C$18*GiaDinh!$C$17</f>
-        <v>64.259999999999991</v>
+        <v>66.10799999999999</v>
       </c>
       <c r="H153" s="7">
         <v>12</v>

</xml_diff>